<commit_message>
Mise a jour du 07-09-2026  9:53:50.54
</commit_message>
<xml_diff>
--- a/contenu/Revision Premiere.xlsx
+++ b/contenu/Revision Premiere.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\Autres ordinateurs\Mon ordinateur portable\Cours\Site\contenu\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maxence\Documents\Cours\Site\contenu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6B21741-4777-40E3-895B-77528FF3DFA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17629EAB-3A9F-4A18-9B37-81D01AD45C0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="14370" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Liste" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="62">
   <si>
     <t>Préfixe</t>
   </si>
@@ -196,16 +196,40 @@
   </si>
   <si>
     <t>R1.SF1.1</t>
+  </si>
+  <si>
+    <t>Calculer les racines d'un polynome du 2nd degrès</t>
+  </si>
+  <si>
+    <t>Factoriser un polynome du 2nd degrès</t>
+  </si>
+  <si>
+    <t>Mettre un polynome du 2nd degrès sous forme canonique</t>
+  </si>
+  <si>
+    <t>Dériver une fonction</t>
+  </si>
+  <si>
+    <t>Dériver un produit</t>
+  </si>
+  <si>
+    <t>dériver un quotient</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -522,27 +546,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:U21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.23046875" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="2.921875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="4.61328125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="4.4609375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="3.15234375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="44.07421875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="3.3046875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="2.88671875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="4.6640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="4.44140625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="3.109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="44.109375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="3.33203125" style="1" customWidth="1"/>
     <col min="8" max="8" width="7" style="1" customWidth="1"/>
-    <col min="10" max="10" width="2.3046875" style="1" customWidth="1"/>
-    <col min="11" max="11" width="3.921875" style="1" customWidth="1"/>
-    <col min="13" max="13" width="1.921875" style="1" customWidth="1"/>
-    <col min="14" max="14" width="2.765625" style="1" customWidth="1"/>
-    <col min="16" max="16" width="2.3828125" style="1" customWidth="1"/>
-    <col min="17" max="17" width="2.3046875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="2.33203125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="3.88671875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="1.88671875" style="1" customWidth="1"/>
+    <col min="14" max="14" width="2.77734375" style="1" customWidth="1"/>
+    <col min="16" max="17" width="2.33203125" style="1" customWidth="1"/>
     <col min="19" max="19" width="2" style="1" customWidth="1"/>
-    <col min="20" max="20" width="2.23046875" style="1" customWidth="1"/>
-    <col min="21" max="21" width="18.23046875" style="1" customWidth="1"/>
+    <col min="20" max="20" width="2.21875" style="1" customWidth="1"/>
+    <col min="21" max="21" width="18.21875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -607,7 +630,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -642,7 +665,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="3" spans="1:21" ht="43.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:21" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -678,7 +701,7 @@
       </c>
       <c r="O3" s="3"/>
     </row>
-    <row r="4" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -713,57 +736,143 @@
         <v>840</v>
       </c>
     </row>
-    <row r="5" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" s="1">
+        <v>2</v>
+      </c>
+      <c r="C5" s="1">
+        <v>1</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>56</v>
+      </c>
       <c r="F5" s="3"/>
       <c r="I5" s="3"/>
       <c r="L5" s="3"/>
     </row>
-    <row r="6" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="1">
+        <v>2</v>
+      </c>
+      <c r="C6" s="1">
+        <v>2</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>57</v>
+      </c>
       <c r="F6" s="3"/>
       <c r="I6" s="3"/>
       <c r="L6" s="3"/>
     </row>
-    <row r="7" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="1">
+        <v>2</v>
+      </c>
+      <c r="C7" s="1">
+        <v>3</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>58</v>
+      </c>
       <c r="I7" s="3"/>
       <c r="L7" s="3"/>
     </row>
-    <row r="8" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="1">
+        <v>3</v>
+      </c>
+      <c r="C8" s="1">
+        <v>1</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>59</v>
+      </c>
       <c r="L8" s="3"/>
     </row>
-    <row r="11" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9" s="1">
+        <v>3</v>
+      </c>
+      <c r="C9" s="1">
+        <v>2</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="1">
+        <v>3</v>
+      </c>
+      <c r="C10" s="1">
+        <v>3</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>21</v>
+      </c>
       <c r="F11" s="3"/>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
     </row>
-    <row r="12" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>21</v>
+      </c>
       <c r="F12" s="3"/>
     </row>
-    <row r="13" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>21</v>
+      </c>
       <c r="F13" s="3"/>
       <c r="I13" s="3"/>
     </row>
-    <row r="14" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F14" s="3"/>
       <c r="I14" s="3"/>
       <c r="L14" s="3"/>
     </row>
-    <row r="15" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F15" s="3"/>
       <c r="I15" s="3"/>
       <c r="L15" s="3"/>
       <c r="O15" s="3"/>
       <c r="R15" s="3"/>
     </row>
-    <row r="19" spans="6:15" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="6:15" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F19" s="3"/>
       <c r="I19" s="3"/>
       <c r="L19" s="3"/>
       <c r="O19" s="3"/>
     </row>
-    <row r="21" spans="6:15" ht="43.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="6:15" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F21" s="3"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -771,16 +880,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:IC230"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.07421875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="11.109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="60" style="1" customWidth="1"/>
-    <col min="3" max="237" width="2.69140625" style="1" customWidth="1"/>
-    <col min="238" max="238" width="11.07421875" style="1" customWidth="1"/>
-    <col min="239" max="16384" width="11.07421875" style="1"/>
+    <col min="3" max="237" width="2.6640625" style="1" customWidth="1"/>
+    <col min="238" max="238" width="11.109375" style="1" customWidth="1"/>
+    <col min="239" max="16384" width="11.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:237" ht="59.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:237" ht="59.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -1493,7 +1602,7 @@
         <v>46570</v>
       </c>
     </row>
-    <row r="2" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>55</v>
       </c>
@@ -1511,7 +1620,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>54</v>
       </c>
@@ -1529,7 +1638,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>30</v>
       </c>
@@ -1547,682 +1656,682 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:237" x14ac:dyDescent="0.3">
       <c r="H5" s="2"/>
     </row>
-    <row r="6" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:237" x14ac:dyDescent="0.3">
       <c r="H6" s="2"/>
     </row>
-    <row r="7" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:237" x14ac:dyDescent="0.3">
       <c r="H7" s="2"/>
     </row>
-    <row r="8" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:237" x14ac:dyDescent="0.3">
       <c r="H8" s="2"/>
     </row>
-    <row r="9" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:237" x14ac:dyDescent="0.3">
       <c r="H9" s="2"/>
     </row>
-    <row r="10" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:237" x14ac:dyDescent="0.3">
       <c r="H10" s="2"/>
     </row>
-    <row r="11" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:237" x14ac:dyDescent="0.3">
       <c r="H11" s="2"/>
     </row>
-    <row r="12" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:237" x14ac:dyDescent="0.3">
       <c r="H12" s="2"/>
     </row>
-    <row r="13" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:237" x14ac:dyDescent="0.3">
       <c r="H13" s="2"/>
     </row>
-    <row r="14" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:237" x14ac:dyDescent="0.3">
       <c r="H14" s="2"/>
     </row>
-    <row r="15" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:237" x14ac:dyDescent="0.3">
       <c r="H15" s="2"/>
     </row>
-    <row r="16" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:237" x14ac:dyDescent="0.3">
       <c r="H16" s="2"/>
     </row>
-    <row r="17" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="17" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H17" s="2"/>
     </row>
-    <row r="18" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="18" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H18" s="2"/>
     </row>
-    <row r="19" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="19" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H19" s="2"/>
     </row>
-    <row r="20" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="20" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H20" s="2"/>
     </row>
-    <row r="21" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="21" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H21" s="2"/>
     </row>
-    <row r="22" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="22" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H22" s="2"/>
     </row>
-    <row r="23" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="23" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H23" s="2"/>
     </row>
-    <row r="24" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="24" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H24" s="2"/>
     </row>
-    <row r="25" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="25" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H25" s="2"/>
     </row>
-    <row r="26" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="26" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H26" s="2"/>
     </row>
-    <row r="27" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="27" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H27" s="2"/>
     </row>
-    <row r="28" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="28" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H28" s="2"/>
     </row>
-    <row r="29" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="29" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H29" s="2"/>
     </row>
-    <row r="30" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="30" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H30" s="2"/>
     </row>
-    <row r="31" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="31" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H31" s="2"/>
     </row>
-    <row r="32" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="32" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H32" s="2"/>
     </row>
-    <row r="33" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="33" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H33" s="2"/>
     </row>
-    <row r="34" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="34" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H34" s="2"/>
     </row>
-    <row r="35" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="35" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H35" s="2"/>
     </row>
-    <row r="36" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="36" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H36" s="2"/>
     </row>
-    <row r="37" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="37" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H37" s="2"/>
     </row>
-    <row r="38" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="38" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H38" s="2"/>
     </row>
-    <row r="39" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="39" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H39" s="2"/>
     </row>
-    <row r="40" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="40" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H40" s="2"/>
     </row>
-    <row r="41" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="41" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H41" s="2"/>
     </row>
-    <row r="42" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="42" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H42" s="2"/>
     </row>
-    <row r="43" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="43" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H43" s="2"/>
     </row>
-    <row r="44" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="44" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H44" s="2"/>
     </row>
-    <row r="45" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="45" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H45" s="2"/>
     </row>
-    <row r="46" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="46" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H46" s="2"/>
     </row>
-    <row r="47" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="47" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H47" s="2"/>
     </row>
-    <row r="48" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="48" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H48" s="2"/>
     </row>
-    <row r="49" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="49" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H49" s="2"/>
     </row>
-    <row r="50" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="50" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H50" s="2"/>
     </row>
-    <row r="51" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="51" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H51" s="2"/>
     </row>
-    <row r="52" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="52" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H52" s="2"/>
     </row>
-    <row r="53" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="53" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H53" s="2"/>
     </row>
-    <row r="54" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="54" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H54" s="2"/>
     </row>
-    <row r="55" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="55" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H55" s="2"/>
     </row>
-    <row r="56" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="56" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H56" s="2"/>
     </row>
-    <row r="57" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="57" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H57" s="2"/>
     </row>
-    <row r="58" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="58" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H58" s="2"/>
     </row>
-    <row r="59" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="59" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H59" s="2"/>
     </row>
-    <row r="60" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="60" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H60" s="2"/>
     </row>
-    <row r="61" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="61" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H61" s="2"/>
     </row>
-    <row r="62" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="62" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H62" s="2"/>
     </row>
-    <row r="63" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="63" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H63" s="2"/>
     </row>
-    <row r="64" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="64" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H64" s="2"/>
     </row>
-    <row r="65" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="65" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H65" s="2"/>
     </row>
-    <row r="66" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="66" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H66" s="2"/>
     </row>
-    <row r="67" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="67" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H67" s="2"/>
     </row>
-    <row r="68" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="68" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H68" s="2"/>
     </row>
-    <row r="69" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="69" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H69" s="2"/>
     </row>
-    <row r="70" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="70" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H70" s="2"/>
     </row>
-    <row r="71" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="71" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H71" s="2"/>
     </row>
-    <row r="72" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="72" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H72" s="2"/>
     </row>
-    <row r="73" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="73" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H73" s="2"/>
     </row>
-    <row r="74" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="74" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H74" s="2"/>
     </row>
-    <row r="75" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="75" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H75" s="2"/>
     </row>
-    <row r="76" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="76" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H76" s="2"/>
     </row>
-    <row r="77" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="77" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H77" s="2"/>
     </row>
-    <row r="78" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="78" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H78" s="2"/>
     </row>
-    <row r="79" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="79" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H79" s="2"/>
     </row>
-    <row r="80" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="80" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H80" s="2"/>
     </row>
-    <row r="81" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="81" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H81" s="2"/>
     </row>
-    <row r="82" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="82" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H82" s="2"/>
     </row>
-    <row r="83" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="83" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H83" s="2"/>
     </row>
-    <row r="84" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="84" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H84" s="2"/>
     </row>
-    <row r="85" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="85" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H85" s="2"/>
     </row>
-    <row r="86" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="86" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H86" s="2"/>
     </row>
-    <row r="87" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="87" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H87" s="2"/>
     </row>
-    <row r="88" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="88" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H88" s="2"/>
     </row>
-    <row r="89" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="89" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H89" s="2"/>
     </row>
-    <row r="90" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="90" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H90" s="2"/>
     </row>
-    <row r="91" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="91" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H91" s="2"/>
     </row>
-    <row r="92" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="92" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H92" s="2"/>
     </row>
-    <row r="93" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="93" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H93" s="2"/>
     </row>
-    <row r="94" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="94" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H94" s="2"/>
     </row>
-    <row r="95" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="95" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H95" s="2"/>
     </row>
-    <row r="96" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="96" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H96" s="2"/>
     </row>
-    <row r="97" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="97" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H97" s="2"/>
     </row>
-    <row r="98" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="98" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H98" s="2"/>
     </row>
-    <row r="99" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="99" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H99" s="2"/>
     </row>
-    <row r="100" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="100" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H100" s="2"/>
     </row>
-    <row r="101" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="101" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H101" s="2"/>
     </row>
-    <row r="102" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="102" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H102" s="2"/>
     </row>
-    <row r="103" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="103" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H103" s="2"/>
     </row>
-    <row r="104" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="104" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H104" s="2"/>
     </row>
-    <row r="105" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="105" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H105" s="2"/>
     </row>
-    <row r="106" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="106" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H106" s="2"/>
     </row>
-    <row r="107" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="107" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H107" s="2"/>
     </row>
-    <row r="108" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="108" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H108" s="2"/>
     </row>
-    <row r="109" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="109" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H109" s="2"/>
     </row>
-    <row r="110" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="110" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H110" s="2"/>
     </row>
-    <row r="111" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="111" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H111" s="2"/>
     </row>
-    <row r="112" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="112" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H112" s="2"/>
     </row>
-    <row r="113" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="113" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H113" s="2"/>
     </row>
-    <row r="114" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="114" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H114" s="2"/>
     </row>
-    <row r="115" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="115" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H115" s="2"/>
     </row>
-    <row r="116" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="116" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H116" s="2"/>
     </row>
-    <row r="117" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="117" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H117" s="2"/>
     </row>
-    <row r="118" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="118" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H118" s="2"/>
     </row>
-    <row r="119" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="119" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H119" s="2"/>
     </row>
-    <row r="120" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="120" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H120" s="2"/>
     </row>
-    <row r="121" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="121" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H121" s="2"/>
     </row>
-    <row r="122" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="122" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H122" s="2"/>
     </row>
-    <row r="123" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="123" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H123" s="2"/>
     </row>
-    <row r="124" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="124" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H124" s="2"/>
     </row>
-    <row r="125" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="125" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H125" s="2"/>
     </row>
-    <row r="126" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="126" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H126" s="2"/>
     </row>
-    <row r="127" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="127" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H127" s="2"/>
     </row>
-    <row r="128" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="128" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H128" s="2"/>
     </row>
-    <row r="129" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="129" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H129" s="2"/>
     </row>
-    <row r="130" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="130" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H130" s="2"/>
     </row>
-    <row r="131" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="131" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H131" s="2"/>
     </row>
-    <row r="132" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="132" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H132" s="2"/>
     </row>
-    <row r="133" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="133" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H133" s="2"/>
     </row>
-    <row r="134" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="134" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H134" s="2"/>
     </row>
-    <row r="135" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="135" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H135" s="2"/>
     </row>
-    <row r="136" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="136" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H136" s="2"/>
     </row>
-    <row r="137" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="137" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H137" s="2"/>
     </row>
-    <row r="138" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="138" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H138" s="2"/>
     </row>
-    <row r="139" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="139" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H139" s="2"/>
     </row>
-    <row r="140" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="140" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H140" s="2"/>
     </row>
-    <row r="141" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="141" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H141" s="2"/>
     </row>
-    <row r="142" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="142" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H142" s="2"/>
     </row>
-    <row r="143" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="143" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H143" s="2"/>
     </row>
-    <row r="144" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="144" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H144" s="2"/>
     </row>
-    <row r="145" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="145" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H145" s="2"/>
     </row>
-    <row r="146" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="146" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H146" s="2"/>
     </row>
-    <row r="147" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="147" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H147" s="2"/>
     </row>
-    <row r="148" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="148" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H148" s="2"/>
     </row>
-    <row r="149" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="149" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H149" s="2"/>
     </row>
-    <row r="150" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="150" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H150" s="2"/>
     </row>
-    <row r="151" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="151" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H151" s="2"/>
     </row>
-    <row r="152" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="152" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H152" s="2"/>
     </row>
-    <row r="153" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="153" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H153" s="2"/>
     </row>
-    <row r="154" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="154" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H154" s="2"/>
     </row>
-    <row r="155" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="155" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H155" s="2"/>
     </row>
-    <row r="156" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="156" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H156" s="2"/>
     </row>
-    <row r="157" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="157" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H157" s="2"/>
     </row>
-    <row r="158" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="158" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H158" s="2"/>
     </row>
-    <row r="159" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="159" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H159" s="2"/>
     </row>
-    <row r="160" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="160" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H160" s="2"/>
     </row>
-    <row r="161" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="161" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H161" s="2"/>
     </row>
-    <row r="162" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="162" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H162" s="2"/>
     </row>
-    <row r="163" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="163" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H163" s="2"/>
     </row>
-    <row r="164" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="164" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H164" s="2"/>
     </row>
-    <row r="165" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="165" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H165" s="2"/>
     </row>
-    <row r="166" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="166" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H166" s="2"/>
     </row>
-    <row r="167" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="167" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H167" s="2"/>
     </row>
-    <row r="168" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="168" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H168" s="2"/>
     </row>
-    <row r="169" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="169" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H169" s="2"/>
     </row>
-    <row r="170" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="170" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H170" s="2"/>
     </row>
-    <row r="171" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="171" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H171" s="2"/>
     </row>
-    <row r="172" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="172" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H172" s="2"/>
     </row>
-    <row r="173" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="173" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H173" s="2"/>
     </row>
-    <row r="174" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="174" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H174" s="2"/>
     </row>
-    <row r="175" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="175" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H175" s="2"/>
     </row>
-    <row r="176" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="176" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H176" s="2"/>
     </row>
-    <row r="177" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="177" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H177" s="2"/>
     </row>
-    <row r="178" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="178" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H178" s="2"/>
     </row>
-    <row r="179" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="179" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H179" s="2"/>
     </row>
-    <row r="180" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="180" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H180" s="2"/>
     </row>
-    <row r="181" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="181" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H181" s="2"/>
     </row>
-    <row r="182" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="182" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H182" s="2"/>
     </row>
-    <row r="183" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="183" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H183" s="2"/>
     </row>
-    <row r="184" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="184" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H184" s="2"/>
     </row>
-    <row r="185" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="185" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H185" s="2"/>
     </row>
-    <row r="186" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="186" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H186" s="2"/>
     </row>
-    <row r="187" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="187" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H187" s="2"/>
     </row>
-    <row r="188" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="188" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H188" s="2"/>
     </row>
-    <row r="189" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="189" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H189" s="2"/>
     </row>
-    <row r="190" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="190" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H190" s="2"/>
     </row>
-    <row r="191" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="191" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H191" s="2"/>
     </row>
-    <row r="192" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="192" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H192" s="2"/>
     </row>
-    <row r="193" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="193" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H193" s="2"/>
     </row>
-    <row r="194" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="194" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H194" s="2"/>
     </row>
-    <row r="195" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="195" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H195" s="2"/>
     </row>
-    <row r="196" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="196" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H196" s="2"/>
     </row>
-    <row r="197" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="197" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H197" s="2"/>
     </row>
-    <row r="198" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="198" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H198" s="2"/>
     </row>
-    <row r="199" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="199" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H199" s="2"/>
     </row>
-    <row r="200" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="200" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H200" s="2"/>
     </row>
-    <row r="201" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="201" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H201" s="2"/>
     </row>
-    <row r="202" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="202" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H202" s="2"/>
     </row>
-    <row r="203" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="203" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H203" s="2"/>
     </row>
-    <row r="204" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="204" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H204" s="2"/>
     </row>
-    <row r="205" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="205" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H205" s="2"/>
     </row>
-    <row r="206" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="206" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H206" s="2"/>
     </row>
-    <row r="207" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="207" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H207" s="2"/>
     </row>
-    <row r="208" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="208" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H208" s="2"/>
     </row>
-    <row r="209" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="209" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H209" s="2"/>
     </row>
-    <row r="210" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="210" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H210" s="2"/>
     </row>
-    <row r="211" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="211" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H211" s="2"/>
     </row>
-    <row r="212" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="212" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H212" s="2"/>
     </row>
-    <row r="213" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="213" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H213" s="2"/>
     </row>
-    <row r="214" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="214" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H214" s="2"/>
     </row>
-    <row r="215" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="215" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H215" s="2"/>
     </row>
-    <row r="216" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="216" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H216" s="2"/>
     </row>
-    <row r="217" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="217" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H217" s="2"/>
     </row>
-    <row r="218" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="218" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H218" s="2"/>
     </row>
-    <row r="219" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="219" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H219" s="2"/>
     </row>
-    <row r="220" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="220" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H220" s="2"/>
     </row>
-    <row r="221" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="221" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H221" s="2"/>
     </row>
-    <row r="222" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="222" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H222" s="2"/>
     </row>
-    <row r="223" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="223" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H223" s="2"/>
     </row>
-    <row r="224" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="224" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H224" s="2"/>
     </row>
-    <row r="225" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="225" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H225" s="2"/>
     </row>
-    <row r="226" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="226" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H226" s="2"/>
     </row>
-    <row r="227" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="227" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H227" s="2"/>
     </row>
-    <row r="228" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="228" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H228" s="2"/>
     </row>
-    <row r="229" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="229" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H229" s="2"/>
     </row>
-    <row r="230" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="230" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H230" s="2"/>
     </row>
   </sheetData>
@@ -2233,12 +2342,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:AQ16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="43" width="3.69140625" style="1" customWidth="1"/>
+    <col min="2" max="43" width="3.6640625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:43" x14ac:dyDescent="0.3">
       <c r="B1">
         <v>37</v>
       </c>
@@ -2366,77 +2475,77 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="7" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="9" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="10" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="11" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="12" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="13" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="14" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="15" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="16" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>51</v>
       </c>
@@ -2449,9 +2558,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B45"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>52</v>
       </c>
@@ -2459,7 +2568,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>36</v>
       </c>
@@ -2467,7 +2576,7 @@
         <v>46266</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>37</v>
       </c>
@@ -2475,7 +2584,7 @@
         <v>46272</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>38</v>
       </c>
@@ -2483,7 +2592,7 @@
         <v>46279</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>39</v>
       </c>
@@ -2491,7 +2600,7 @@
         <v>46286</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>40</v>
       </c>
@@ -2499,7 +2608,7 @@
         <v>46293</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>41</v>
       </c>
@@ -2507,7 +2616,7 @@
         <v>46300</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>42</v>
       </c>
@@ -2515,7 +2624,7 @@
         <v>46307</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>43</v>
       </c>
@@ -2523,7 +2632,7 @@
         <v>46314</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>44</v>
       </c>
@@ -2531,7 +2640,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>45</v>
       </c>
@@ -2539,7 +2648,7 @@
         <v>46328</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>46</v>
       </c>
@@ -2547,7 +2656,7 @@
         <v>46335</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>47</v>
       </c>
@@ -2555,7 +2664,7 @@
         <v>46342</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>48</v>
       </c>
@@ -2563,7 +2672,7 @@
         <v>46349</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>49</v>
       </c>
@@ -2571,7 +2680,7 @@
         <v>46356</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>50</v>
       </c>
@@ -2579,7 +2688,7 @@
         <v>46363</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>51</v>
       </c>
@@ -2587,7 +2696,7 @@
         <v>46370</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>52</v>
       </c>
@@ -2595,7 +2704,7 @@
         <v>46377</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>53</v>
       </c>
@@ -2603,7 +2712,7 @@
         <v>46384</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>1</v>
       </c>
@@ -2611,7 +2720,7 @@
         <v>46391</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>2</v>
       </c>
@@ -2619,7 +2728,7 @@
         <v>46398</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>3</v>
       </c>
@@ -2627,7 +2736,7 @@
         <v>46405</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>4</v>
       </c>
@@ -2635,7 +2744,7 @@
         <v>46412</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>5</v>
       </c>
@@ -2643,7 +2752,7 @@
         <v>46419</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>6</v>
       </c>
@@ -2651,7 +2760,7 @@
         <v>46426</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>7</v>
       </c>
@@ -2659,7 +2768,7 @@
         <v>46433</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>8</v>
       </c>
@@ -2667,7 +2776,7 @@
         <v>46440</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>9</v>
       </c>
@@ -2675,7 +2784,7 @@
         <v>46447</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>10</v>
       </c>
@@ -2683,7 +2792,7 @@
         <v>46454</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>11</v>
       </c>
@@ -2691,7 +2800,7 @@
         <v>46461</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>12</v>
       </c>
@@ -2699,7 +2808,7 @@
         <v>46468</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>13</v>
       </c>
@@ -2707,7 +2816,7 @@
         <v>46475</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>14</v>
       </c>
@@ -2715,7 +2824,7 @@
         <v>46482</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>15</v>
       </c>
@@ -2723,7 +2832,7 @@
         <v>46489</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>16</v>
       </c>
@@ -2731,7 +2840,7 @@
         <v>46496</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>17</v>
       </c>
@@ -2739,7 +2848,7 @@
         <v>46503</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>18</v>
       </c>
@@ -2747,7 +2856,7 @@
         <v>46510</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>19</v>
       </c>
@@ -2755,7 +2864,7 @@
         <v>46517</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>20</v>
       </c>
@@ -2763,7 +2872,7 @@
         <v>46524</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>21</v>
       </c>
@@ -2771,7 +2880,7 @@
         <v>46531</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>22</v>
       </c>
@@ -2779,7 +2888,7 @@
         <v>46538</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>23</v>
       </c>
@@ -2787,7 +2896,7 @@
         <v>46545</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>24</v>
       </c>
@@ -2795,7 +2904,7 @@
         <v>46552</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>25</v>
       </c>
@@ -2803,7 +2912,7 @@
         <v>46559</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>26</v>
       </c>

</xml_diff>

<commit_message>
Mise a jour du 08-09-2026 13:20:35.32
</commit_message>
<xml_diff>
--- a/contenu/Revision Premiere.xlsx
+++ b/contenu/Revision Premiere.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maxence\Documents\Cours\Site\contenu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8D2726F-E495-48AC-831D-80ECD32B4243}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C5F2BB6-ADC7-402F-B439-DF9BD03AD98C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -791,8 +791,14 @@
       <c r="F5" s="3" t="s">
         <v>39</v>
       </c>
+      <c r="H5">
+        <v>517</v>
+      </c>
       <c r="I5" s="3" t="s">
         <v>40</v>
+      </c>
+      <c r="K5">
+        <v>779</v>
       </c>
       <c r="L5" s="3"/>
     </row>
@@ -815,6 +821,9 @@
       <c r="F6" s="3" t="s">
         <v>43</v>
       </c>
+      <c r="H6">
+        <v>367</v>
+      </c>
       <c r="I6" s="3"/>
       <c r="L6" s="3"/>
     </row>
@@ -837,6 +846,9 @@
       <c r="F7" t="s">
         <v>46</v>
       </c>
+      <c r="H7">
+        <v>604</v>
+      </c>
       <c r="I7" s="3"/>
       <c r="L7" s="3"/>
     </row>
@@ -894,6 +906,9 @@
       <c r="F10" t="s">
         <v>53</v>
       </c>
+      <c r="H10">
+        <v>813</v>
+      </c>
     </row>
     <row r="11" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
@@ -914,7 +929,9 @@
       <c r="F11" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="H11" s="3"/>
+      <c r="H11" s="3">
+        <v>697</v>
+      </c>
       <c r="I11" s="3"/>
     </row>
     <row r="12" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
@@ -964,8 +981,8 @@
     <col min="1" max="1" width="11.109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="49.33203125" style="1" customWidth="1"/>
     <col min="3" max="237" width="2.6640625" style="1" customWidth="1"/>
-    <col min="238" max="239" width="11.109375" style="1" customWidth="1"/>
-    <col min="240" max="16384" width="11.109375" style="1"/>
+    <col min="238" max="240" width="11.109375" style="1" customWidth="1"/>
+    <col min="241" max="16384" width="11.109375" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:237" ht="59.1" customHeight="1" x14ac:dyDescent="0.3">
@@ -1692,10 +1709,9 @@
       <c r="W2" t="s">
         <v>57</v>
       </c>
-      <c r="Z2" s="1" t="s">
+      <c r="Z2" t="s">
         <v>57</v>
       </c>
-      <c r="AA2"/>
     </row>
     <row r="3" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
@@ -1708,10 +1724,9 @@
       <c r="W3" t="s">
         <v>57</v>
       </c>
-      <c r="Y3" s="1" t="s">
+      <c r="Y3" t="s">
         <v>57</v>
       </c>
-      <c r="Z3"/>
     </row>
     <row r="4" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
@@ -1721,14 +1736,13 @@
         <v>33</v>
       </c>
       <c r="H4" s="2"/>
-      <c r="X4" s="1" t="s">
+      <c r="X4" t="s">
         <v>57</v>
       </c>
-      <c r="Y4"/>
-      <c r="AA4" s="1" t="s">
+      <c r="Z4" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="AB4"/>
+      <c r="AA4"/>
       <c r="AH4" t="s">
         <v>57</v>
       </c>

</xml_diff>

<commit_message>
Mise a jour du 11-09-2026 14:34:09.49
</commit_message>
<xml_diff>
--- a/contenu/Revision Premiere.xlsx
+++ b/contenu/Revision Premiere.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maxence\Documents\Cours\Site\contenu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C5F2BB6-ADC7-402F-B439-DF9BD03AD98C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67B5A92A-5FA9-4F92-8782-344B67DAFD0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="23232" windowHeight="6216" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Liste" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="88">
   <si>
     <t>Préfixe</t>
   </si>
@@ -111,6 +111,9 @@
     <t>7OkCnme--VY</t>
   </si>
   <si>
+    <t>Niv 1 non obligatoire</t>
+  </si>
+  <si>
     <t>R1.SF1.2</t>
   </si>
   <si>
@@ -139,6 +142,39 @@
   </si>
   <si>
     <t>ay-T6EGkM5I</t>
+  </si>
+  <si>
+    <t>R2</t>
+  </si>
+  <si>
+    <t>R2.SF1.4</t>
+  </si>
+  <si>
+    <t>Somme de terme arithmétique</t>
+  </si>
+  <si>
+    <t>XiKVQa8BWko</t>
+  </si>
+  <si>
+    <t>WeDtB9ZUTHs</t>
+  </si>
+  <si>
+    <t>iSfevWwk8e4</t>
+  </si>
+  <si>
+    <t>R3</t>
+  </si>
+  <si>
+    <t>R3.SF1.5</t>
+  </si>
+  <si>
+    <t>Somme de terme géométrique</t>
+  </si>
+  <si>
+    <t>gUkOjvAiZGA</t>
+  </si>
+  <si>
+    <t>OUFkINbcHrI</t>
   </si>
   <si>
     <t>R1.SF2.1</t>
@@ -581,7 +617,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U21"/>
+  <dimension ref="A1:U23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2.88671875" style="1" customWidth="1"/>
@@ -700,6 +736,9 @@
       <c r="N2">
         <v>528</v>
       </c>
+      <c r="U2" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="3" spans="1:21" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
@@ -712,25 +751,25 @@
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H3">
         <v>214</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="K3">
         <v>320</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="N3">
         <v>624</v>
@@ -748,25 +787,25 @@
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H4">
         <v>484</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="K4">
         <v>629</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="N4">
         <v>840</v>
@@ -774,58 +813,68 @@
     </row>
     <row r="5" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="B5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H5">
-        <v>517</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>40</v>
+        <v>401</v>
+      </c>
+      <c r="I5" t="s">
+        <v>42</v>
       </c>
       <c r="K5">
-        <v>779</v>
-      </c>
-      <c r="L5" s="3"/>
+        <v>190</v>
+      </c>
+      <c r="L5" t="s">
+        <v>43</v>
+      </c>
+      <c r="N5">
+        <v>270</v>
+      </c>
     </row>
     <row r="6" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="B6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C6">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D6" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="E6" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="H6">
-        <v>367</v>
+        <v>193</v>
       </c>
       <c r="I6" s="3"/>
-      <c r="L6" s="3"/>
+      <c r="L6" t="s">
+        <v>48</v>
+      </c>
+      <c r="N6">
+        <v>441</v>
+      </c>
     </row>
     <row r="7" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
@@ -835,21 +884,26 @@
         <v>2</v>
       </c>
       <c r="C7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D7" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="E7" t="s">
-        <v>45</v>
-      </c>
-      <c r="F7" t="s">
-        <v>46</v>
+        <v>50</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>51</v>
       </c>
       <c r="H7">
-        <v>604</v>
-      </c>
-      <c r="I7" s="3"/>
+        <v>517</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="K7">
+        <v>779</v>
+      </c>
       <c r="L7" s="3"/>
     </row>
     <row r="8" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
@@ -857,37 +911,52 @@
         <v>21</v>
       </c>
       <c r="B8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D8" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E8" t="s">
-        <v>48</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="H8">
+        <v>367</v>
+      </c>
+      <c r="I8" s="3"/>
       <c r="L8" s="3"/>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>21</v>
       </c>
       <c r="B9">
+        <v>2</v>
+      </c>
+      <c r="C9">
         <v>3</v>
       </c>
-      <c r="C9">
-        <v>2</v>
-      </c>
       <c r="D9" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="E9" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+        <v>57</v>
+      </c>
+      <c r="F9" t="s">
+        <v>58</v>
+      </c>
+      <c r="H9">
+        <v>604</v>
+      </c>
+      <c r="I9" s="3"/>
+      <c r="L9" s="3"/>
+    </row>
+    <row r="10" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -895,22 +964,17 @@
         <v>3</v>
       </c>
       <c r="C10">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D10" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="E10" t="s">
-        <v>52</v>
-      </c>
-      <c r="F10" t="s">
-        <v>53</v>
-      </c>
-      <c r="H10">
-        <v>813</v>
-      </c>
-    </row>
-    <row r="11" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>60</v>
+      </c>
+      <c r="L10" s="3"/>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>21</v>
       </c>
@@ -918,55 +982,95 @@
         <v>3</v>
       </c>
       <c r="C11">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D11" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="E11" t="s">
-        <v>55</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="H11" s="3">
-        <v>697</v>
-      </c>
-      <c r="I11" s="3"/>
-    </row>
-    <row r="12" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>21</v>
       </c>
-      <c r="F12" s="3"/>
+      <c r="B12">
+        <v>3</v>
+      </c>
+      <c r="C12">
+        <v>3</v>
+      </c>
+      <c r="D12" t="s">
+        <v>63</v>
+      </c>
+      <c r="E12" t="s">
+        <v>64</v>
+      </c>
+      <c r="F12" t="s">
+        <v>65</v>
+      </c>
+      <c r="H12">
+        <v>813</v>
+      </c>
     </row>
     <row r="13" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>21</v>
       </c>
-      <c r="F13" s="3"/>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13">
+        <v>4</v>
+      </c>
+      <c r="D13" t="s">
+        <v>66</v>
+      </c>
+      <c r="E13" t="s">
+        <v>67</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="H13" s="3">
+        <v>697</v>
+      </c>
       <c r="I13" s="3"/>
     </row>
     <row r="14" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>21</v>
+      </c>
       <c r="F14" s="3"/>
-      <c r="I14" s="3"/>
-      <c r="L14" s="3"/>
     </row>
     <row r="15" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>21</v>
+      </c>
       <c r="F15" s="3"/>
       <c r="I15" s="3"/>
-      <c r="L15" s="3"/>
-      <c r="O15" s="3"/>
-      <c r="R15" s="3"/>
-    </row>
-    <row r="19" spans="6:15" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F19" s="3"/>
-      <c r="I19" s="3"/>
-      <c r="L19" s="3"/>
-      <c r="O19" s="3"/>
-    </row>
-    <row r="21" spans="6:15" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F16" s="3"/>
+      <c r="I16" s="3"/>
+      <c r="L16" s="3"/>
+    </row>
+    <row r="17" spans="6:18" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F17" s="3"/>
+      <c r="I17" s="3"/>
+      <c r="L17" s="3"/>
+      <c r="O17" s="3"/>
+      <c r="R17" s="3"/>
+    </row>
+    <row r="21" spans="6:18" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F21" s="3"/>
+      <c r="I21" s="3"/>
+      <c r="L21" s="3"/>
+      <c r="O21" s="3"/>
+    </row>
+    <row r="23" spans="6:18" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F23" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -981,8 +1085,8 @@
     <col min="1" max="1" width="11.109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="49.33203125" style="1" customWidth="1"/>
     <col min="3" max="237" width="2.6640625" style="1" customWidth="1"/>
-    <col min="238" max="240" width="11.109375" style="1" customWidth="1"/>
-    <col min="241" max="16384" width="11.109375" style="1"/>
+    <col min="238" max="241" width="11.109375" style="1" customWidth="1"/>
+    <col min="242" max="16384" width="11.109375" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:237" ht="59.1" customHeight="1" x14ac:dyDescent="0.3">
@@ -1707,113 +1811,133 @@
       </c>
       <c r="H2" s="2"/>
       <c r="W2" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="Z2" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H3" s="2"/>
       <c r="W3" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="Y3" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H4" s="2"/>
       <c r="X4" t="s">
-        <v>57</v>
-      </c>
-      <c r="Z4" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="AA4"/>
+        <v>69</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>69</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>69</v>
+      </c>
       <c r="AH4" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H5" s="2"/>
+      <c r="AG5" s="1" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="6" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="B6" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="H6" s="2"/>
+      <c r="AD6" s="1" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="7" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B7" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="H7" s="2"/>
     </row>
     <row r="8" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="B8" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="H8" s="2"/>
     </row>
     <row r="9" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="B9" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="H9" s="2"/>
     </row>
     <row r="10" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="B10" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="H10" s="2"/>
     </row>
     <row r="11" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="B11" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="H11" s="2"/>
     </row>
     <row r="12" spans="1:237" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B12" t="s">
+        <v>64</v>
+      </c>
       <c r="H12" s="2"/>
     </row>
     <row r="13" spans="1:237" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>66</v>
+      </c>
+      <c r="B13" t="s">
+        <v>67</v>
+      </c>
       <c r="H13" s="2"/>
     </row>
     <row r="14" spans="1:237" x14ac:dyDescent="0.3">
@@ -2500,10 +2624,10 @@
         <v>42</v>
       </c>
       <c r="H1" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="I1" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="J1">
         <v>45</v>
@@ -2527,10 +2651,10 @@
         <v>51</v>
       </c>
       <c r="Q1" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="R1" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="S1">
         <v>1</v>
@@ -2551,10 +2675,10 @@
         <v>6</v>
       </c>
       <c r="Y1" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="Z1" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="AA1">
         <v>9</v>
@@ -2575,10 +2699,10 @@
         <v>14</v>
       </c>
       <c r="AG1" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="AH1" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="AI1">
         <v>17</v>
@@ -2610,77 +2734,77 @@
     </row>
     <row r="2" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>60</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>62</v>
+        <v>74</v>
       </c>
     </row>
     <row r="6" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>63</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>64</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>65</v>
+        <v>77</v>
       </c>
     </row>
     <row r="9" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
     </row>
     <row r="10" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>67</v>
+        <v>79</v>
       </c>
     </row>
     <row r="11" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
     </row>
     <row r="12" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>69</v>
+        <v>81</v>
       </c>
     </row>
     <row r="13" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>70</v>
+        <v>82</v>
       </c>
     </row>
     <row r="14" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>71</v>
+        <v>83</v>
       </c>
     </row>
     <row r="15" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>72</v>
+        <v>84</v>
       </c>
     </row>
     <row r="16" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>73</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -2695,10 +2819,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>74</v>
+        <v>86</v>
       </c>
       <c r="B1" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Mise a jour du 21-09-2026 15:49:58.30
</commit_message>
<xml_diff>
--- a/contenu/Revision Premiere.xlsx
+++ b/contenu/Revision Premiere.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maxence\Documents\Cours\Site\contenu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67B5A92A-5FA9-4F92-8782-344B67DAFD0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04F36B1C-F08C-46E8-BCC0-8C88970EFD34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="23232" windowHeight="6216" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Liste" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="99">
   <si>
     <t>Préfixe</t>
   </si>
@@ -235,6 +235,39 @@
   </si>
   <si>
     <t>LwlPq4QyZoo</t>
+  </si>
+  <si>
+    <t>R1.SF4.1</t>
+  </si>
+  <si>
+    <t>Résoudre un système par substitution</t>
+  </si>
+  <si>
+    <t>vXSDO4HNn2c</t>
+  </si>
+  <si>
+    <t>x_AJ6vtBXms</t>
+  </si>
+  <si>
+    <t>R1.SF4.2</t>
+  </si>
+  <si>
+    <t>Résoudre un système par combinaison</t>
+  </si>
+  <si>
+    <t>Zw-qI9DFv54</t>
+  </si>
+  <si>
+    <t>xlcJc2gOg9U</t>
+  </si>
+  <si>
+    <t>R1.SF4.3</t>
+  </si>
+  <si>
+    <t>Résoudre un système par pivot de Gauss</t>
+  </si>
+  <si>
+    <t>LIc0loIdsV0</t>
   </si>
   <si>
     <t>x</t>
@@ -1042,19 +1075,84 @@
       <c r="A14" t="s">
         <v>21</v>
       </c>
-      <c r="F14" s="3"/>
+      <c r="B14">
+        <v>4</v>
+      </c>
+      <c r="C14">
+        <v>1</v>
+      </c>
+      <c r="D14" t="s">
+        <v>69</v>
+      </c>
+      <c r="E14" t="s">
+        <v>70</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="H14">
+        <v>280</v>
+      </c>
+      <c r="I14" t="s">
+        <v>72</v>
+      </c>
+      <c r="K14">
+        <v>319</v>
+      </c>
     </row>
     <row r="15" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>21</v>
       </c>
-      <c r="F15" s="3"/>
-      <c r="I15" s="3"/>
+      <c r="B15">
+        <v>4</v>
+      </c>
+      <c r="C15">
+        <v>2</v>
+      </c>
+      <c r="D15" t="s">
+        <v>73</v>
+      </c>
+      <c r="E15" t="s">
+        <v>74</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="H15">
+        <v>409</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="K15">
+        <v>277</v>
+      </c>
     </row>
     <row r="16" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16">
+        <v>4</v>
+      </c>
+      <c r="C16">
+        <v>3</v>
+      </c>
+      <c r="D16" t="s">
+        <v>77</v>
+      </c>
+      <c r="E16" t="s">
+        <v>78</v>
+      </c>
       <c r="F16" s="3"/>
       <c r="I16" s="3"/>
-      <c r="L16" s="3"/>
+      <c r="L16" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="N16">
+        <v>901</v>
+      </c>
     </row>
     <row r="17" spans="6:18" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F17" s="3"/>
@@ -1085,8 +1183,8 @@
     <col min="1" max="1" width="11.109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="49.33203125" style="1" customWidth="1"/>
     <col min="3" max="237" width="2.6640625" style="1" customWidth="1"/>
-    <col min="238" max="241" width="11.109375" style="1" customWidth="1"/>
-    <col min="242" max="16384" width="11.109375" style="1"/>
+    <col min="238" max="242" width="11.109375" style="1" customWidth="1"/>
+    <col min="243" max="16384" width="11.109375" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:237" ht="59.1" customHeight="1" x14ac:dyDescent="0.3">
@@ -1811,10 +1909,10 @@
       </c>
       <c r="H2" s="2"/>
       <c r="W2" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="Z2" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:237" x14ac:dyDescent="0.3">
@@ -1826,10 +1924,10 @@
       </c>
       <c r="H3" s="2"/>
       <c r="W3" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="Y3" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4" spans="1:237" x14ac:dyDescent="0.3">
@@ -1841,16 +1939,16 @@
       </c>
       <c r="H4" s="2"/>
       <c r="X4" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="Z4" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="AB4" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="AH4" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
     </row>
     <row r="5" spans="1:237" x14ac:dyDescent="0.3">
@@ -1861,8 +1959,8 @@
         <v>40</v>
       </c>
       <c r="H5" s="2"/>
-      <c r="AG5" s="1" t="s">
-        <v>69</v>
+      <c r="AG5" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="6" spans="1:237" x14ac:dyDescent="0.3">
@@ -1873,8 +1971,8 @@
         <v>46</v>
       </c>
       <c r="H6" s="2"/>
-      <c r="AD6" s="1" t="s">
-        <v>69</v>
+      <c r="AD6" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="7" spans="1:237" x14ac:dyDescent="0.3">
@@ -1941,13 +2039,49 @@
       <c r="H13" s="2"/>
     </row>
     <row r="14" spans="1:237" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>69</v>
+      </c>
+      <c r="B14" t="s">
+        <v>70</v>
+      </c>
       <c r="H14" s="2"/>
+      <c r="AH14" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="AL14" s="1" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="15" spans="1:237" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>73</v>
+      </c>
+      <c r="B15" t="s">
+        <v>74</v>
+      </c>
       <c r="H15" s="2"/>
+      <c r="AI15" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="AJ15" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="AL15" s="1" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="16" spans="1:237" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>77</v>
+      </c>
+      <c r="B16" t="s">
+        <v>78</v>
+      </c>
       <c r="H16" s="2"/>
+      <c r="AI16" s="1" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="17" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H17" s="2"/>
@@ -2624,10 +2758,10 @@
         <v>42</v>
       </c>
       <c r="H1" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="I1" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="J1">
         <v>45</v>
@@ -2651,10 +2785,10 @@
         <v>51</v>
       </c>
       <c r="Q1" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="R1" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="S1">
         <v>1</v>
@@ -2675,10 +2809,10 @@
         <v>6</v>
       </c>
       <c r="Y1" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="Z1" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="AA1">
         <v>9</v>
@@ -2699,10 +2833,10 @@
         <v>14</v>
       </c>
       <c r="AG1" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="AH1" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="AI1">
         <v>17</v>
@@ -2734,77 +2868,77 @@
     </row>
     <row r="2" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>74</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>75</v>
+        <v>86</v>
       </c>
     </row>
     <row r="7" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>76</v>
+        <v>87</v>
       </c>
     </row>
     <row r="8" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>77</v>
+        <v>88</v>
       </c>
     </row>
     <row r="9" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>78</v>
+        <v>89</v>
       </c>
     </row>
     <row r="10" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>79</v>
+        <v>90</v>
       </c>
     </row>
     <row r="11" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>80</v>
+        <v>91</v>
       </c>
     </row>
     <row r="12" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
     </row>
     <row r="13" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
     </row>
     <row r="14" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
     </row>
     <row r="15" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
     </row>
     <row r="16" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>85</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -2819,10 +2953,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>86</v>
+        <v>97</v>
       </c>
       <c r="B1" t="s">
-        <v>87</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Mise a jour du 21-09-2026 18:43:40.08
</commit_message>
<xml_diff>
--- a/contenu/Revision Premiere.xlsx
+++ b/contenu/Revision Premiere.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maxence\Documents\Cours\Site\contenu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04F36B1C-F08C-46E8-BCC0-8C88970EFD34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D108692A-10C0-4868-8162-FF7213A998D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="99">
   <si>
     <t>Préfixe</t>
   </si>
@@ -1947,9 +1947,7 @@
       <c r="AB4" t="s">
         <v>80</v>
       </c>
-      <c r="AH4" t="s">
-        <v>80</v>
-      </c>
+      <c r="AH4"/>
     </row>
     <row r="5" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
@@ -2046,7 +2044,7 @@
         <v>70</v>
       </c>
       <c r="H14" s="2"/>
-      <c r="AH14" s="1" t="s">
+      <c r="AJ14" s="1" t="s">
         <v>80</v>
       </c>
       <c r="AL14" s="1" t="s">
@@ -2064,7 +2062,7 @@
       <c r="AI15" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="AJ15" s="1" t="s">
+      <c r="AK15" s="1" t="s">
         <v>80</v>
       </c>
       <c r="AL15" s="1" t="s">

</xml_diff>

<commit_message>
Mise a jour du 25-09-2026  7:56:43.33
</commit_message>
<xml_diff>
--- a/contenu/Revision Premiere.xlsx
+++ b/contenu/Revision Premiere.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maxence\Documents\Cours\Site\contenu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5AB63C6-0B6C-4588-A0ED-A3BE55056F79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B5B237C-BF3B-4F37-A4D1-B920818737FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="99">
   <si>
     <t>Préfixe</t>
   </si>
@@ -1914,6 +1914,9 @@
       <c r="Z2" t="s">
         <v>80</v>
       </c>
+      <c r="AL2" s="1" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="3" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
@@ -1929,6 +1932,9 @@
       <c r="Y3" t="s">
         <v>80</v>
       </c>
+      <c r="AL3" s="1" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="4" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
@@ -1948,6 +1954,9 @@
         <v>80</v>
       </c>
       <c r="AH4"/>
+      <c r="AL4" s="1" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="5" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
@@ -2047,9 +2056,6 @@
       <c r="AJ14" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="AL14" s="1" t="s">
-        <v>80</v>
-      </c>
     </row>
     <row r="15" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
@@ -2063,9 +2069,6 @@
         <v>80</v>
       </c>
       <c r="AK15" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="AL15" s="1" t="s">
         <v>80</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise a jour du 06-10-2026 12:12:12,90
</commit_message>
<xml_diff>
--- a/contenu/Revision Premiere.xlsx
+++ b/contenu/Revision Premiere.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Liste" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Plannification" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Calendrier" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="liste date semaine" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Liste" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plannification" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calendrier" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="liste date semaine" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -402,23 +402,23 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:U24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.21875" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.23046875" defaultRowHeight="14.6"/>
   <cols>
-    <col width="2.88671875" customWidth="1" style="1" min="1" max="1"/>
-    <col width="4.6640625" customWidth="1" style="1" min="2" max="2"/>
-    <col width="4.44140625" customWidth="1" style="1" min="3" max="3"/>
-    <col width="3.109375" customWidth="1" style="1" min="4" max="4"/>
-    <col width="44.109375" customWidth="1" style="1" min="5" max="5"/>
-    <col width="3.33203125" customWidth="1" style="1" min="7" max="7"/>
+    <col width="2.84375" customWidth="1" style="1" min="1" max="1"/>
+    <col width="4.69140625" customWidth="1" style="1" min="2" max="2"/>
+    <col width="4.4609375" customWidth="1" style="1" min="3" max="3"/>
+    <col width="3.07421875" customWidth="1" style="1" min="4" max="4"/>
+    <col width="44.07421875" customWidth="1" style="1" min="5" max="5"/>
+    <col width="3.3046875" customWidth="1" style="1" min="7" max="7"/>
     <col width="7" customWidth="1" style="1" min="8" max="8"/>
-    <col width="2.33203125" customWidth="1" style="1" min="10" max="10"/>
-    <col width="3.88671875" customWidth="1" style="1" min="11" max="11"/>
-    <col width="1.88671875" customWidth="1" style="1" min="13" max="13"/>
-    <col width="2.77734375" customWidth="1" style="1" min="14" max="14"/>
-    <col width="2.33203125" customWidth="1" style="1" min="16" max="17"/>
+    <col width="2.3046875" customWidth="1" style="1" min="10" max="10"/>
+    <col width="3.84375" customWidth="1" style="1" min="11" max="11"/>
+    <col width="1.84375" customWidth="1" style="1" min="13" max="13"/>
+    <col width="2.765625" customWidth="1" style="1" min="14" max="14"/>
+    <col width="2.3046875" customWidth="1" style="1" min="16" max="17"/>
     <col width="2" customWidth="1" style="1" min="19" max="19"/>
-    <col width="2.21875" customWidth="1" style="1" min="20" max="20"/>
-    <col width="18.21875" customWidth="1" style="1" min="21" max="21"/>
+    <col width="2.23046875" customWidth="1" style="1" min="20" max="20"/>
+    <col width="18.23046875" customWidth="1" style="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -528,7 +528,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="29.1" customHeight="1" s="1">
+    <row r="2" ht="29.15" customHeight="1" s="1">
       <c r="A2" t="inlineStr">
         <is>
           <t>R1</t>
@@ -580,7 +580,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="43.8" customHeight="1" s="1">
+    <row r="3" ht="43.85" customHeight="1" s="1">
       <c r="A3" t="inlineStr">
         <is>
           <t>R1</t>
@@ -628,7 +628,7 @@
       </c>
       <c r="O3" s="3" t="n"/>
     </row>
-    <row r="4" ht="29.1" customHeight="1" s="1">
+    <row r="4" ht="29.15" customHeight="1" s="1">
       <c r="A4" t="inlineStr">
         <is>
           <t>R1</t>
@@ -675,7 +675,7 @@
         <v>840</v>
       </c>
     </row>
-    <row r="5" ht="29.1" customHeight="1" s="1">
+    <row r="5" ht="29.15" customHeight="1" s="1">
       <c r="A5" t="inlineStr">
         <is>
           <t>R2</t>
@@ -722,7 +722,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="6" ht="29.1" customHeight="1" s="1">
+    <row r="6" ht="29.15" customHeight="1" s="1">
       <c r="A6" t="inlineStr">
         <is>
           <t>R3</t>
@@ -762,7 +762,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="7" ht="29.1" customHeight="1" s="1">
+    <row r="7" ht="29.15" customHeight="1" s="1">
       <c r="A7" t="inlineStr">
         <is>
           <t>R1</t>
@@ -802,7 +802,7 @@
       </c>
       <c r="L7" s="3" t="n"/>
     </row>
-    <row r="8" ht="29.1" customHeight="1" s="1">
+    <row r="8" ht="29.15" customHeight="1" s="1">
       <c r="A8" t="inlineStr">
         <is>
           <t>R1</t>
@@ -835,7 +835,7 @@
       <c r="I8" s="3" t="n"/>
       <c r="L8" s="3" t="n"/>
     </row>
-    <row r="9" ht="29.1" customHeight="1" s="1">
+    <row r="9" ht="29.15" customHeight="1" s="1">
       <c r="A9" t="inlineStr">
         <is>
           <t>R1</t>
@@ -868,7 +868,7 @@
       <c r="I9" s="3" t="n"/>
       <c r="L9" s="3" t="n"/>
     </row>
-    <row r="10" ht="29.1" customHeight="1" s="1">
+    <row r="10" ht="29.15" customHeight="1" s="1">
       <c r="A10" t="inlineStr">
         <is>
           <t>R1</t>
@@ -930,6 +930,14 @@
       <c r="H11" t="n">
         <v>336</v>
       </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>MZauKTHZcUI</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>483</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -962,7 +970,7 @@
         <v>813</v>
       </c>
     </row>
-    <row r="13" s="1">
+    <row r="13">
       <c r="A13" t="inlineStr">
         <is>
           <t>R1</t>
@@ -992,8 +1000,24 @@
       <c r="H13" t="n">
         <v>225</v>
       </c>
-    </row>
-    <row r="14" ht="29.1" customHeight="1" s="1">
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>fvD2OK3HphQ</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>698</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>fvD2OK3HphQ</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="14" ht="29.15" customHeight="1" s="1">
       <c r="A14" t="inlineStr">
         <is>
           <t>R1</t>
@@ -1025,7 +1049,7 @@
       </c>
       <c r="I14" s="3" t="n"/>
     </row>
-    <row r="15" ht="29.1" customHeight="1" s="1">
+    <row r="15" ht="29.15" customHeight="1" s="1">
       <c r="A15" t="inlineStr">
         <is>
           <t>R1</t>
@@ -1064,7 +1088,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="16" ht="29.1" customHeight="1" s="1">
+    <row r="16" ht="29.15" customHeight="1" s="1">
       <c r="A16" t="inlineStr">
         <is>
           <t>R1</t>
@@ -1103,7 +1127,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="17" ht="29.1" customHeight="1" s="1">
+    <row r="17" ht="29.15" customHeight="1" s="1">
       <c r="A17" t="inlineStr">
         <is>
           <t>R1</t>
@@ -1136,7 +1160,7 @@
         <v>901</v>
       </c>
     </row>
-    <row r="18" ht="29.1" customHeight="1" s="1">
+    <row r="18" ht="29.15" customHeight="1" s="1">
       <c r="F18" s="3" t="n"/>
       <c r="I18" s="3" t="n"/>
       <c r="L18" s="3" t="n"/>
@@ -1146,14 +1170,14 @@
     <row r="19"/>
     <row r="20"/>
     <row r="21"/>
-    <row r="22" ht="29.1" customHeight="1" s="1">
+    <row r="22" ht="29.15" customHeight="1" s="1">
       <c r="F22" s="3" t="n"/>
       <c r="I22" s="3" t="n"/>
       <c r="L22" s="3" t="n"/>
       <c r="O22" s="3" t="n"/>
     </row>
     <row r="23"/>
-    <row r="24" ht="43.8" customHeight="1" s="1">
+    <row r="24" ht="43.85" customHeight="1" s="1">
       <c r="F24" s="3" t="n"/>
     </row>
   </sheetData>
@@ -1168,16 +1192,16 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:IC230"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.109375" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.07421875" defaultRowHeight="14.6"/>
   <cols>
-    <col width="11.109375" customWidth="1" style="1" min="1" max="1"/>
-    <col width="49.33203125" customWidth="1" style="1" min="2" max="2"/>
-    <col width="2.6640625" customWidth="1" style="1" min="3" max="237"/>
-    <col width="11.109375" customWidth="1" style="1" min="238" max="242"/>
-    <col width="11.109375" customWidth="1" style="1" min="243" max="16384"/>
+    <col width="11.07421875" customWidth="1" style="1" min="1" max="1"/>
+    <col width="49.3046875" customWidth="1" style="1" min="2" max="2"/>
+    <col width="2.69140625" customWidth="1" style="1" min="3" max="237"/>
+    <col width="11.07421875" customWidth="1" style="1" min="238" max="243"/>
+    <col width="11.07421875" customWidth="1" style="1" min="244" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" ht="59.1" customHeight="1" s="1">
+    <row r="1" ht="59.15" customHeight="1" s="1">
       <c r="A1" t="inlineStr">
         <is>
           <t>Code</t>
@@ -2124,6 +2148,11 @@
         </is>
       </c>
       <c r="H13" s="2" t="n"/>
+      <c r="AS13" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2848,9 +2877,9 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AQ16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6"/>
   <cols>
-    <col width="3.6640625" customWidth="1" style="1" min="2" max="43"/>
+    <col width="3.69140625" customWidth="1" style="1" min="2" max="43"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3114,7 +3143,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B45"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">

</xml_diff>

<commit_message>
Mise a jour du 12-10-2026 15:22:23.61
</commit_message>
<xml_diff>
--- a/contenu/Revision Premiere.xlsx
+++ b/contenu/Revision Premiere.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\Autres ordinateurs\Mon ordinateur portable\Cours\Site\contenu\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maxence\Documents\Cours\Site\contenu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50BD43D1-8A63-4A02-BE15-7FC8EC5F8F07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AF7A442-6AA2-4464-9CAE-A5342C509F80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Liste" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="127">
   <si>
     <t>Préfixe</t>
   </si>
@@ -288,13 +288,52 @@
     <t>R1.SF5.1</t>
   </si>
   <si>
+    <t>Opérations sur des exponentielles</t>
+  </si>
+  <si>
+    <t>mAzQ5f_UTcs</t>
+  </si>
+  <si>
+    <t>47Y814hMtC0</t>
+  </si>
+  <si>
+    <t>R1.SF5.2</t>
+  </si>
+  <si>
+    <t>Factoriser avec exponentielle</t>
+  </si>
+  <si>
+    <t>7sltvZDKl1E</t>
+  </si>
+  <si>
+    <t>oY6QSwsFeqk</t>
+  </si>
+  <si>
+    <t>gvHvNSrIB-A</t>
+  </si>
+  <si>
+    <t>R1.SF5.3</t>
+  </si>
+  <si>
     <t>Résoudre une équation avec exponentielle</t>
   </si>
   <si>
     <t>y5GfPIZqOCM</t>
   </si>
   <si>
-    <t>R1.SF5.2</t>
+    <t>R1.SF5.4</t>
+  </si>
+  <si>
+    <t>Signe d'expression avec exponentielle</t>
+  </si>
+  <si>
+    <t>dnQYNEM1Yag</t>
+  </si>
+  <si>
+    <t>L_yU82P1cgg</t>
+  </si>
+  <si>
+    <t>R1.SF5.5</t>
   </si>
   <si>
     <t>Dériver et variation avec exponentielle</t>
@@ -306,10 +345,10 @@
     <t>rhCKIwUN3Ps</t>
   </si>
   <si>
+    <t>uVj7Utq-7Bo</t>
+  </si>
+  <si>
     <t>Niv1 : ne pas faire f</t>
-  </si>
-  <si>
-    <t>R1.SF5.3</t>
   </si>
   <si>
     <t>x</t>
@@ -695,27 +734,27 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.23046875" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:U24"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="2.84375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="4.69140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="4.4609375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="10.4609375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="44.07421875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="3.3046875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="2.88671875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="4.6640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="4.44140625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="10.44140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="44.109375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="3.33203125" style="1" customWidth="1"/>
     <col min="8" max="8" width="7" style="1" customWidth="1"/>
-    <col min="10" max="10" width="2.3046875" style="1" customWidth="1"/>
-    <col min="11" max="11" width="3.84375" style="1" customWidth="1"/>
-    <col min="13" max="13" width="1.84375" style="1" customWidth="1"/>
-    <col min="14" max="14" width="2.765625" style="1" customWidth="1"/>
-    <col min="16" max="17" width="2.3046875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="2.33203125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="3.88671875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="1.88671875" style="1" customWidth="1"/>
+    <col min="14" max="14" width="2.77734375" style="1" customWidth="1"/>
+    <col min="16" max="17" width="2.33203125" style="1" customWidth="1"/>
     <col min="19" max="19" width="2" style="1" customWidth="1"/>
-    <col min="20" max="20" width="2.23046875" style="1" customWidth="1"/>
-    <col min="21" max="21" width="18.23046875" style="1" customWidth="1"/>
+    <col min="20" max="20" width="2.21875" style="1" customWidth="1"/>
+    <col min="21" max="21" width="18.21875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -780,7 +819,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -818,7 +857,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:21" ht="43.85" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:21" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -854,7 +893,7 @@
       </c>
       <c r="O3" s="3"/>
     </row>
-    <row r="4" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -889,7 +928,7 @@
         <v>840</v>
       </c>
     </row>
-    <row r="5" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>38</v>
       </c>
@@ -924,7 +963,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="6" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>44</v>
       </c>
@@ -954,7 +993,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="7" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -984,7 +1023,7 @@
       </c>
       <c r="L7" s="3"/>
     </row>
-    <row r="8" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -1009,7 +1048,7 @@
       <c r="I8" s="3"/>
       <c r="L8" s="3"/>
     </row>
-    <row r="9" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -1034,7 +1073,7 @@
       <c r="I9" s="3"/>
       <c r="L9" s="3"/>
     </row>
-    <row r="10" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -1064,7 +1103,7 @@
       </c>
       <c r="L10" s="3"/>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>21</v>
       </c>
@@ -1093,7 +1132,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -1116,7 +1155,7 @@
         <v>813</v>
       </c>
     </row>
-    <row r="13" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>21</v>
       </c>
@@ -1145,7 +1184,7 @@
         <v>698</v>
       </c>
     </row>
-    <row r="14" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>21</v>
       </c>
@@ -1174,7 +1213,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="15" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>21</v>
       </c>
@@ -1203,7 +1242,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="16" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>21</v>
       </c>
@@ -1228,7 +1267,7 @@
         <v>901</v>
       </c>
     </row>
-    <row r="17" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>21</v>
       </c>
@@ -1248,14 +1287,16 @@
         <v>87</v>
       </c>
       <c r="H17">
-        <v>306</v>
-      </c>
-      <c r="I17" s="3"/>
-      <c r="L17" s="3"/>
-      <c r="O17" s="3"/>
-      <c r="R17" s="3"/>
-    </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.4">
+        <v>152</v>
+      </c>
+      <c r="I17" t="s">
+        <v>88</v>
+      </c>
+      <c r="K17">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="18" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>21</v>
       </c>
@@ -1266,34 +1307,31 @@
         <v>2</v>
       </c>
       <c r="D18" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E18" t="s">
-        <v>89</v>
-      </c>
-      <c r="F18" t="s">
         <v>90</v>
       </c>
+      <c r="F18" s="3" t="s">
+        <v>91</v>
+      </c>
       <c r="H18">
-        <v>379</v>
+        <v>102</v>
       </c>
       <c r="I18" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K18">
-        <v>509</v>
-      </c>
-      <c r="L18" t="s">
-        <v>66</v>
-      </c>
-      <c r="N18">
-        <v>483</v>
-      </c>
-      <c r="U18" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.4">
+        <v>185</v>
+      </c>
+      <c r="R18" t="s">
+        <v>93</v>
+      </c>
+      <c r="T18">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="19" spans="1:21" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>21</v>
       </c>
@@ -1304,39 +1342,116 @@
         <v>3</v>
       </c>
       <c r="D19" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.4">
+        <v>94</v>
+      </c>
+      <c r="E19" t="s">
+        <v>95</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="H19">
+        <v>306</v>
+      </c>
+      <c r="L19" s="3"/>
+      <c r="O19" s="3"/>
+      <c r="R19" s="3"/>
+    </row>
+    <row r="20" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>21</v>
       </c>
       <c r="B20">
         <v>5</v>
       </c>
-    </row>
-    <row r="21" spans="1:21" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C20">
+        <v>4</v>
+      </c>
+      <c r="D20" t="s">
+        <v>97</v>
+      </c>
+      <c r="E20" t="s">
+        <v>98</v>
+      </c>
+      <c r="F20" t="s">
+        <v>99</v>
+      </c>
+      <c r="H20">
+        <v>219</v>
+      </c>
+      <c r="I20" t="s">
+        <v>100</v>
+      </c>
+      <c r="K20">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="21" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>21</v>
       </c>
-      <c r="F21" s="3"/>
-      <c r="I21" s="3"/>
-      <c r="L21" s="3"/>
-      <c r="O21" s="3"/>
-    </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.4">
+      <c r="B21">
+        <v>5</v>
+      </c>
+      <c r="C21">
+        <v>5</v>
+      </c>
+      <c r="D21" t="s">
+        <v>101</v>
+      </c>
+      <c r="E21" t="s">
+        <v>102</v>
+      </c>
+      <c r="F21" t="s">
+        <v>103</v>
+      </c>
+      <c r="H21">
+        <v>379</v>
+      </c>
+      <c r="I21" t="s">
+        <v>104</v>
+      </c>
+      <c r="K21">
+        <v>509</v>
+      </c>
+      <c r="L21" t="s">
+        <v>66</v>
+      </c>
+      <c r="N21">
+        <v>483</v>
+      </c>
+      <c r="O21" t="s">
+        <v>105</v>
+      </c>
+      <c r="Q21">
+        <v>493</v>
+      </c>
+      <c r="U21" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="22" spans="1:21" ht="29.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>21</v>
       </c>
-      <c r="B22">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="23" spans="1:21" ht="43.85" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="F22" s="3"/>
+      <c r="I22" s="3"/>
+      <c r="L22" s="3"/>
+      <c r="O22" s="3"/>
+    </row>
+    <row r="23" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>21</v>
       </c>
-      <c r="F23" s="3"/>
+      <c r="B23">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:21" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>21</v>
+      </c>
+      <c r="F24" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1346,16 +1461,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:IC230"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.07421875" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.07421875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="49.3046875" style="1" customWidth="1"/>
-    <col min="3" max="237" width="2.69140625" style="1" customWidth="1"/>
-    <col min="238" max="246" width="11.07421875" style="1" customWidth="1"/>
-    <col min="247" max="16384" width="11.07421875" style="1"/>
+    <col min="1" max="1" width="11.109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="49.33203125" style="1" customWidth="1"/>
+    <col min="3" max="237" width="2.6640625" style="1" customWidth="1"/>
+    <col min="238" max="248" width="11.109375" style="1" customWidth="1"/>
+    <col min="249" max="16384" width="11.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:237" ht="59.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:237" ht="59.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -2068,7 +2183,7 @@
         <v>46570</v>
       </c>
     </row>
-    <row r="2" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>22</v>
       </c>
@@ -2077,16 +2192,16 @@
       </c>
       <c r="H2" s="2"/>
       <c r="W2" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="Z2" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="AL2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="3" spans="1:237" x14ac:dyDescent="0.4">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="3" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>28</v>
       </c>
@@ -2095,16 +2210,16 @@
       </c>
       <c r="H3" s="2"/>
       <c r="W3" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="Y3" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="AL3" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="4" spans="1:237" x14ac:dyDescent="0.4">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="4" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>33</v>
       </c>
@@ -2113,19 +2228,19 @@
       </c>
       <c r="H4" s="2"/>
       <c r="X4" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="Z4" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="AB4" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="AL4" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="5" spans="1:237" x14ac:dyDescent="0.4">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="5" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>39</v>
       </c>
@@ -2134,10 +2249,10 @@
       </c>
       <c r="H5" s="2"/>
       <c r="AG5" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="6" spans="1:237" x14ac:dyDescent="0.4">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="6" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>45</v>
       </c>
@@ -2146,10 +2261,10 @@
       </c>
       <c r="H6" s="2"/>
       <c r="AD6" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="7" spans="1:237" x14ac:dyDescent="0.4">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="7" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>49</v>
       </c>
@@ -2157,11 +2272,11 @@
         <v>50</v>
       </c>
       <c r="H7" s="2"/>
-      <c r="AX7" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="8" spans="1:237" x14ac:dyDescent="0.4">
+      <c r="AX7" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="8" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>53</v>
       </c>
@@ -2169,11 +2284,11 @@
         <v>54</v>
       </c>
       <c r="H8" s="2"/>
-      <c r="AX8" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="9" spans="1:237" x14ac:dyDescent="0.4">
+      <c r="AX8" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="9" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>56</v>
       </c>
@@ -2182,7 +2297,7 @@
       </c>
       <c r="H9" s="2"/>
     </row>
-    <row r="10" spans="1:237" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>59</v>
       </c>
@@ -2191,10 +2306,10 @@
       </c>
       <c r="H10" s="2"/>
       <c r="AS10" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="11" spans="1:237" x14ac:dyDescent="0.4">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="11" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>63</v>
       </c>
@@ -2203,10 +2318,10 @@
       </c>
       <c r="H11" s="2"/>
       <c r="AT11" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="12" spans="1:237" x14ac:dyDescent="0.4">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="12" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>67</v>
       </c>
@@ -2215,25 +2330,25 @@
       </c>
       <c r="H12" s="2"/>
       <c r="AT12" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="13" spans="1:237" x14ac:dyDescent="0.4">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="13" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>70</v>
       </c>
       <c r="B13" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="H13" s="2"/>
       <c r="AS13" t="s">
-        <v>94</v>
-      </c>
-      <c r="AY13" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="14" spans="1:237" x14ac:dyDescent="0.4">
+        <v>107</v>
+      </c>
+      <c r="AY13" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="14" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>74</v>
       </c>
@@ -2242,10 +2357,10 @@
       </c>
       <c r="H14" s="2"/>
       <c r="AJ14" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="15" spans="1:237" x14ac:dyDescent="0.4">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="15" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>78</v>
       </c>
@@ -2254,13 +2369,13 @@
       </c>
       <c r="H15" s="2"/>
       <c r="AI15" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="AK15" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="16" spans="1:237" x14ac:dyDescent="0.4">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="16" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>82</v>
       </c>
@@ -2269,10 +2384,10 @@
       </c>
       <c r="H16" s="2"/>
       <c r="AI16" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="17" spans="1:49" x14ac:dyDescent="0.4">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="17" spans="1:51" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>85</v>
       </c>
@@ -2280,659 +2395,683 @@
         <v>86</v>
       </c>
       <c r="H17" s="2"/>
-      <c r="AW17" s="1" t="s">
+      <c r="AW17" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="18" spans="1:51" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>89</v>
+      </c>
+      <c r="B18" t="s">
+        <v>90</v>
+      </c>
+      <c r="H18" s="2"/>
+      <c r="AW18" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="19" spans="1:51" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="18" spans="1:49" x14ac:dyDescent="0.4">
-      <c r="A18" t="s">
-        <v>88</v>
-      </c>
-      <c r="B18" t="s">
-        <v>89</v>
-      </c>
-      <c r="H18" s="2"/>
-      <c r="AW18" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="19" spans="1:49" x14ac:dyDescent="0.4">
-      <c r="A19" t="s">
-        <v>93</v>
+      <c r="B19" t="s">
+        <v>95</v>
       </c>
       <c r="H19" s="2"/>
-    </row>
-    <row r="20" spans="1:49" x14ac:dyDescent="0.4">
+      <c r="AX19" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="20" spans="1:51" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>97</v>
+      </c>
+      <c r="B20" t="s">
+        <v>98</v>
+      </c>
       <c r="H20" s="2"/>
-    </row>
-    <row r="21" spans="1:49" x14ac:dyDescent="0.4">
+      <c r="AY20" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="21" spans="1:51" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>101</v>
+      </c>
+      <c r="B21" t="s">
+        <v>102</v>
+      </c>
       <c r="H21" s="2"/>
-    </row>
-    <row r="22" spans="1:49" x14ac:dyDescent="0.4">
+      <c r="AY21" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="22" spans="1:51" x14ac:dyDescent="0.3">
       <c r="H22" s="2"/>
     </row>
-    <row r="23" spans="1:49" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:51" x14ac:dyDescent="0.3">
       <c r="H23" s="2"/>
     </row>
-    <row r="24" spans="1:49" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:51" x14ac:dyDescent="0.3">
       <c r="H24" s="2"/>
     </row>
-    <row r="25" spans="1:49" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:51" x14ac:dyDescent="0.3">
       <c r="H25" s="2"/>
     </row>
-    <row r="26" spans="1:49" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:51" x14ac:dyDescent="0.3">
       <c r="H26" s="2"/>
     </row>
-    <row r="27" spans="1:49" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:51" x14ac:dyDescent="0.3">
       <c r="H27" s="2"/>
     </row>
-    <row r="28" spans="1:49" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:51" x14ac:dyDescent="0.3">
       <c r="H28" s="2"/>
     </row>
-    <row r="29" spans="1:49" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:51" x14ac:dyDescent="0.3">
       <c r="H29" s="2"/>
     </row>
-    <row r="30" spans="1:49" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:51" x14ac:dyDescent="0.3">
       <c r="H30" s="2"/>
     </row>
-    <row r="31" spans="1:49" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:51" x14ac:dyDescent="0.3">
       <c r="H31" s="2"/>
     </row>
-    <row r="32" spans="1:49" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:51" x14ac:dyDescent="0.3">
       <c r="H32" s="2"/>
     </row>
-    <row r="33" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="33" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H33" s="2"/>
     </row>
-    <row r="34" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="34" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H34" s="2"/>
     </row>
-    <row r="35" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="35" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H35" s="2"/>
     </row>
-    <row r="36" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="36" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H36" s="2"/>
     </row>
-    <row r="37" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="37" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H37" s="2"/>
     </row>
-    <row r="38" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="38" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H38" s="2"/>
     </row>
-    <row r="39" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="39" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H39" s="2"/>
     </row>
-    <row r="40" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="40" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H40" s="2"/>
     </row>
-    <row r="41" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="41" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H41" s="2"/>
     </row>
-    <row r="42" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="42" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H42" s="2"/>
     </row>
-    <row r="43" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="43" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H43" s="2"/>
     </row>
-    <row r="44" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="44" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H44" s="2"/>
     </row>
-    <row r="45" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="45" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H45" s="2"/>
     </row>
-    <row r="46" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="46" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H46" s="2"/>
     </row>
-    <row r="47" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="47" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H47" s="2"/>
     </row>
-    <row r="48" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="48" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H48" s="2"/>
     </row>
-    <row r="49" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="49" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H49" s="2"/>
     </row>
-    <row r="50" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="50" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H50" s="2"/>
     </row>
-    <row r="51" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="51" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H51" s="2"/>
     </row>
-    <row r="52" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="52" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H52" s="2"/>
     </row>
-    <row r="53" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="53" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H53" s="2"/>
     </row>
-    <row r="54" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="54" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H54" s="2"/>
     </row>
-    <row r="55" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="55" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H55" s="2"/>
     </row>
-    <row r="56" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="56" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H56" s="2"/>
     </row>
-    <row r="57" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="57" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H57" s="2"/>
     </row>
-    <row r="58" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="58" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H58" s="2"/>
     </row>
-    <row r="59" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="59" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H59" s="2"/>
     </row>
-    <row r="60" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="60" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H60" s="2"/>
     </row>
-    <row r="61" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="61" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H61" s="2"/>
     </row>
-    <row r="62" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="62" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H62" s="2"/>
     </row>
-    <row r="63" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="63" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H63" s="2"/>
     </row>
-    <row r="64" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="64" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H64" s="2"/>
     </row>
-    <row r="65" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="65" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H65" s="2"/>
     </row>
-    <row r="66" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="66" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H66" s="2"/>
     </row>
-    <row r="67" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="67" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H67" s="2"/>
     </row>
-    <row r="68" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="68" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H68" s="2"/>
     </row>
-    <row r="69" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="69" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H69" s="2"/>
     </row>
-    <row r="70" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="70" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H70" s="2"/>
     </row>
-    <row r="71" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="71" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H71" s="2"/>
     </row>
-    <row r="72" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="72" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H72" s="2"/>
     </row>
-    <row r="73" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="73" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H73" s="2"/>
     </row>
-    <row r="74" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="74" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H74" s="2"/>
     </row>
-    <row r="75" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="75" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H75" s="2"/>
     </row>
-    <row r="76" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="76" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H76" s="2"/>
     </row>
-    <row r="77" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="77" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H77" s="2"/>
     </row>
-    <row r="78" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="78" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H78" s="2"/>
     </row>
-    <row r="79" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="79" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H79" s="2"/>
     </row>
-    <row r="80" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="80" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H80" s="2"/>
     </row>
-    <row r="81" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="81" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H81" s="2"/>
     </row>
-    <row r="82" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="82" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H82" s="2"/>
     </row>
-    <row r="83" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="83" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H83" s="2"/>
     </row>
-    <row r="84" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="84" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H84" s="2"/>
     </row>
-    <row r="85" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="85" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H85" s="2"/>
     </row>
-    <row r="86" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="86" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H86" s="2"/>
     </row>
-    <row r="87" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="87" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H87" s="2"/>
     </row>
-    <row r="88" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="88" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H88" s="2"/>
     </row>
-    <row r="89" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="89" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H89" s="2"/>
     </row>
-    <row r="90" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="90" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H90" s="2"/>
     </row>
-    <row r="91" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="91" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H91" s="2"/>
     </row>
-    <row r="92" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="92" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H92" s="2"/>
     </row>
-    <row r="93" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="93" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H93" s="2"/>
     </row>
-    <row r="94" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="94" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H94" s="2"/>
     </row>
-    <row r="95" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="95" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H95" s="2"/>
     </row>
-    <row r="96" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="96" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H96" s="2"/>
     </row>
-    <row r="97" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="97" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H97" s="2"/>
     </row>
-    <row r="98" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="98" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H98" s="2"/>
     </row>
-    <row r="99" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="99" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H99" s="2"/>
     </row>
-    <row r="100" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="100" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H100" s="2"/>
     </row>
-    <row r="101" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="101" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H101" s="2"/>
     </row>
-    <row r="102" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="102" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H102" s="2"/>
     </row>
-    <row r="103" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="103" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H103" s="2"/>
     </row>
-    <row r="104" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="104" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H104" s="2"/>
     </row>
-    <row r="105" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="105" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H105" s="2"/>
     </row>
-    <row r="106" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="106" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H106" s="2"/>
     </row>
-    <row r="107" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="107" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H107" s="2"/>
     </row>
-    <row r="108" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="108" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H108" s="2"/>
     </row>
-    <row r="109" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="109" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H109" s="2"/>
     </row>
-    <row r="110" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="110" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H110" s="2"/>
     </row>
-    <row r="111" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="111" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H111" s="2"/>
     </row>
-    <row r="112" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="112" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H112" s="2"/>
     </row>
-    <row r="113" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="113" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H113" s="2"/>
     </row>
-    <row r="114" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="114" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H114" s="2"/>
     </row>
-    <row r="115" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="115" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H115" s="2"/>
     </row>
-    <row r="116" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="116" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H116" s="2"/>
     </row>
-    <row r="117" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="117" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H117" s="2"/>
     </row>
-    <row r="118" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="118" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H118" s="2"/>
     </row>
-    <row r="119" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="119" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H119" s="2"/>
     </row>
-    <row r="120" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="120" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H120" s="2"/>
     </row>
-    <row r="121" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="121" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H121" s="2"/>
     </row>
-    <row r="122" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="122" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H122" s="2"/>
     </row>
-    <row r="123" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="123" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H123" s="2"/>
     </row>
-    <row r="124" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="124" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H124" s="2"/>
     </row>
-    <row r="125" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="125" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H125" s="2"/>
     </row>
-    <row r="126" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="126" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H126" s="2"/>
     </row>
-    <row r="127" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="127" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H127" s="2"/>
     </row>
-    <row r="128" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="128" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H128" s="2"/>
     </row>
-    <row r="129" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="129" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H129" s="2"/>
     </row>
-    <row r="130" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="130" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H130" s="2"/>
     </row>
-    <row r="131" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="131" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H131" s="2"/>
     </row>
-    <row r="132" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="132" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H132" s="2"/>
     </row>
-    <row r="133" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="133" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H133" s="2"/>
     </row>
-    <row r="134" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="134" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H134" s="2"/>
     </row>
-    <row r="135" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="135" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H135" s="2"/>
     </row>
-    <row r="136" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="136" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H136" s="2"/>
     </row>
-    <row r="137" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="137" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H137" s="2"/>
     </row>
-    <row r="138" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="138" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H138" s="2"/>
     </row>
-    <row r="139" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="139" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H139" s="2"/>
     </row>
-    <row r="140" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="140" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H140" s="2"/>
     </row>
-    <row r="141" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="141" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H141" s="2"/>
     </row>
-    <row r="142" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="142" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H142" s="2"/>
     </row>
-    <row r="143" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="143" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H143" s="2"/>
     </row>
-    <row r="144" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="144" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H144" s="2"/>
     </row>
-    <row r="145" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="145" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H145" s="2"/>
     </row>
-    <row r="146" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="146" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H146" s="2"/>
     </row>
-    <row r="147" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="147" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H147" s="2"/>
     </row>
-    <row r="148" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="148" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H148" s="2"/>
     </row>
-    <row r="149" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="149" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H149" s="2"/>
     </row>
-    <row r="150" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="150" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H150" s="2"/>
     </row>
-    <row r="151" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="151" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H151" s="2"/>
     </row>
-    <row r="152" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="152" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H152" s="2"/>
     </row>
-    <row r="153" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="153" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H153" s="2"/>
     </row>
-    <row r="154" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="154" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H154" s="2"/>
     </row>
-    <row r="155" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="155" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H155" s="2"/>
     </row>
-    <row r="156" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="156" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H156" s="2"/>
     </row>
-    <row r="157" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="157" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H157" s="2"/>
     </row>
-    <row r="158" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="158" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H158" s="2"/>
     </row>
-    <row r="159" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="159" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H159" s="2"/>
     </row>
-    <row r="160" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="160" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H160" s="2"/>
     </row>
-    <row r="161" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="161" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H161" s="2"/>
     </row>
-    <row r="162" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="162" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H162" s="2"/>
     </row>
-    <row r="163" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="163" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H163" s="2"/>
     </row>
-    <row r="164" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="164" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H164" s="2"/>
     </row>
-    <row r="165" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="165" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H165" s="2"/>
     </row>
-    <row r="166" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="166" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H166" s="2"/>
     </row>
-    <row r="167" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="167" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H167" s="2"/>
     </row>
-    <row r="168" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="168" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H168" s="2"/>
     </row>
-    <row r="169" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="169" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H169" s="2"/>
     </row>
-    <row r="170" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="170" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H170" s="2"/>
     </row>
-    <row r="171" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="171" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H171" s="2"/>
     </row>
-    <row r="172" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="172" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H172" s="2"/>
     </row>
-    <row r="173" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="173" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H173" s="2"/>
     </row>
-    <row r="174" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="174" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H174" s="2"/>
     </row>
-    <row r="175" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="175" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H175" s="2"/>
     </row>
-    <row r="176" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="176" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H176" s="2"/>
     </row>
-    <row r="177" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="177" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H177" s="2"/>
     </row>
-    <row r="178" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="178" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H178" s="2"/>
     </row>
-    <row r="179" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="179" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H179" s="2"/>
     </row>
-    <row r="180" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="180" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H180" s="2"/>
     </row>
-    <row r="181" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="181" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H181" s="2"/>
     </row>
-    <row r="182" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="182" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H182" s="2"/>
     </row>
-    <row r="183" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="183" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H183" s="2"/>
     </row>
-    <row r="184" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="184" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H184" s="2"/>
     </row>
-    <row r="185" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="185" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H185" s="2"/>
     </row>
-    <row r="186" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="186" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H186" s="2"/>
     </row>
-    <row r="187" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="187" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H187" s="2"/>
     </row>
-    <row r="188" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="188" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H188" s="2"/>
     </row>
-    <row r="189" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="189" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H189" s="2"/>
     </row>
-    <row r="190" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="190" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H190" s="2"/>
     </row>
-    <row r="191" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="191" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H191" s="2"/>
     </row>
-    <row r="192" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="192" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H192" s="2"/>
     </row>
-    <row r="193" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="193" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H193" s="2"/>
     </row>
-    <row r="194" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="194" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H194" s="2"/>
     </row>
-    <row r="195" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="195" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H195" s="2"/>
     </row>
-    <row r="196" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="196" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H196" s="2"/>
     </row>
-    <row r="197" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="197" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H197" s="2"/>
     </row>
-    <row r="198" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="198" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H198" s="2"/>
     </row>
-    <row r="199" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="199" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H199" s="2"/>
     </row>
-    <row r="200" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="200" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H200" s="2"/>
     </row>
-    <row r="201" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="201" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H201" s="2"/>
     </row>
-    <row r="202" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="202" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H202" s="2"/>
     </row>
-    <row r="203" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="203" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H203" s="2"/>
     </row>
-    <row r="204" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="204" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H204" s="2"/>
     </row>
-    <row r="205" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="205" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H205" s="2"/>
     </row>
-    <row r="206" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="206" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H206" s="2"/>
     </row>
-    <row r="207" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="207" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H207" s="2"/>
     </row>
-    <row r="208" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="208" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H208" s="2"/>
     </row>
-    <row r="209" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="209" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H209" s="2"/>
     </row>
-    <row r="210" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="210" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H210" s="2"/>
     </row>
-    <row r="211" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="211" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H211" s="2"/>
     </row>
-    <row r="212" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="212" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H212" s="2"/>
     </row>
-    <row r="213" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="213" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H213" s="2"/>
     </row>
-    <row r="214" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="214" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H214" s="2"/>
     </row>
-    <row r="215" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="215" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H215" s="2"/>
     </row>
-    <row r="216" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="216" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H216" s="2"/>
     </row>
-    <row r="217" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="217" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H217" s="2"/>
     </row>
-    <row r="218" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="218" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H218" s="2"/>
     </row>
-    <row r="219" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="219" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H219" s="2"/>
     </row>
-    <row r="220" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="220" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H220" s="2"/>
     </row>
-    <row r="221" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="221" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H221" s="2"/>
     </row>
-    <row r="222" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="222" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H222" s="2"/>
     </row>
-    <row r="223" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="223" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H223" s="2"/>
     </row>
-    <row r="224" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="224" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H224" s="2"/>
     </row>
-    <row r="225" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="225" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H225" s="2"/>
     </row>
-    <row r="226" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="226" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H226" s="2"/>
     </row>
-    <row r="227" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="227" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H227" s="2"/>
     </row>
-    <row r="228" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="228" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H228" s="2"/>
     </row>
-    <row r="229" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="229" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H229" s="2"/>
     </row>
-    <row r="230" spans="8:8" x14ac:dyDescent="0.4">
+    <row r="230" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H230" s="2"/>
     </row>
   </sheetData>
@@ -2943,12 +3082,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:AQ16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="43" width="3.69140625" style="1" customWidth="1"/>
+    <col min="2" max="43" width="3.6640625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:43" x14ac:dyDescent="0.3">
       <c r="B1">
         <v>37</v>
       </c>
@@ -2968,10 +3107,10 @@
         <v>42</v>
       </c>
       <c r="H1" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
       <c r="I1" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
       <c r="J1">
         <v>45</v>
@@ -2995,10 +3134,10 @@
         <v>51</v>
       </c>
       <c r="Q1" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
       <c r="R1" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
       <c r="S1">
         <v>1</v>
@@ -3019,10 +3158,10 @@
         <v>6</v>
       </c>
       <c r="Y1" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
       <c r="Z1" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
       <c r="AA1">
         <v>9</v>
@@ -3043,10 +3182,10 @@
         <v>14</v>
       </c>
       <c r="AG1" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
       <c r="AH1" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
       <c r="AI1">
         <v>17</v>
@@ -3076,79 +3215,79 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:43" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="3" spans="1:43" x14ac:dyDescent="0.4">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="3" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="4" spans="1:43" x14ac:dyDescent="0.4">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="4" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="5" spans="1:43" x14ac:dyDescent="0.4">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="5" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="6" spans="1:43" x14ac:dyDescent="0.4">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="6" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="7" spans="1:43" x14ac:dyDescent="0.4">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="7" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="8" spans="1:43" x14ac:dyDescent="0.4">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="8" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="9" spans="1:43" x14ac:dyDescent="0.4">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="9" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="10" spans="1:43" x14ac:dyDescent="0.4">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="10" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="11" spans="1:43" x14ac:dyDescent="0.4">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="11" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="12" spans="1:43" x14ac:dyDescent="0.4">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="12" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="13" spans="1:43" x14ac:dyDescent="0.4">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="13" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="14" spans="1:43" x14ac:dyDescent="0.4">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="14" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="15" spans="1:43" x14ac:dyDescent="0.4">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="15" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="16" spans="1:43" x14ac:dyDescent="0.4">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="16" spans="1:43" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>111</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -3159,17 +3298,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B45"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>112</v>
+        <v>125</v>
       </c>
       <c r="B1" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>36</v>
       </c>
@@ -3177,7 +3316,7 @@
         <v>46266</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>37</v>
       </c>
@@ -3185,7 +3324,7 @@
         <v>46272</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>38</v>
       </c>
@@ -3193,7 +3332,7 @@
         <v>46279</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>39</v>
       </c>
@@ -3201,7 +3340,7 @@
         <v>46286</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>40</v>
       </c>
@@ -3209,7 +3348,7 @@
         <v>46293</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>41</v>
       </c>
@@ -3217,7 +3356,7 @@
         <v>46300</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>42</v>
       </c>
@@ -3225,7 +3364,7 @@
         <v>46307</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>43</v>
       </c>
@@ -3233,7 +3372,7 @@
         <v>46314</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>44</v>
       </c>
@@ -3241,7 +3380,7 @@
         <v>46321</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>45</v>
       </c>
@@ -3249,7 +3388,7 @@
         <v>46328</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>46</v>
       </c>
@@ -3257,7 +3396,7 @@
         <v>46335</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>47</v>
       </c>
@@ -3265,7 +3404,7 @@
         <v>46342</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>48</v>
       </c>
@@ -3273,7 +3412,7 @@
         <v>46349</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>49</v>
       </c>
@@ -3281,7 +3420,7 @@
         <v>46356</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>50</v>
       </c>
@@ -3289,7 +3428,7 @@
         <v>46363</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>51</v>
       </c>
@@ -3297,7 +3436,7 @@
         <v>46370</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>52</v>
       </c>
@@ -3305,7 +3444,7 @@
         <v>46377</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>53</v>
       </c>
@@ -3313,7 +3452,7 @@
         <v>46384</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>1</v>
       </c>
@@ -3321,7 +3460,7 @@
         <v>46391</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>2</v>
       </c>
@@ -3329,7 +3468,7 @@
         <v>46398</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>3</v>
       </c>
@@ -3337,7 +3476,7 @@
         <v>46405</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>4</v>
       </c>
@@ -3345,7 +3484,7 @@
         <v>46412</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>5</v>
       </c>
@@ -3353,7 +3492,7 @@
         <v>46419</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>6</v>
       </c>
@@ -3361,7 +3500,7 @@
         <v>46426</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>7</v>
       </c>
@@ -3369,7 +3508,7 @@
         <v>46433</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>8</v>
       </c>
@@ -3377,7 +3516,7 @@
         <v>46440</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>9</v>
       </c>
@@ -3385,7 +3524,7 @@
         <v>46447</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>10</v>
       </c>
@@ -3393,7 +3532,7 @@
         <v>46454</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>11</v>
       </c>
@@ -3401,7 +3540,7 @@
         <v>46461</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>12</v>
       </c>
@@ -3409,7 +3548,7 @@
         <v>46468</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>13</v>
       </c>
@@ -3417,7 +3556,7 @@
         <v>46475</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>14</v>
       </c>
@@ -3425,7 +3564,7 @@
         <v>46482</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>15</v>
       </c>
@@ -3433,7 +3572,7 @@
         <v>46489</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>16</v>
       </c>
@@ -3441,7 +3580,7 @@
         <v>46496</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>17</v>
       </c>
@@ -3449,7 +3588,7 @@
         <v>46503</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>18</v>
       </c>
@@ -3457,7 +3596,7 @@
         <v>46510</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>19</v>
       </c>
@@ -3465,7 +3604,7 @@
         <v>46517</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>20</v>
       </c>
@@ -3473,7 +3612,7 @@
         <v>46524</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>21</v>
       </c>
@@ -3481,7 +3620,7 @@
         <v>46531</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>22</v>
       </c>
@@ -3489,7 +3628,7 @@
         <v>46538</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>23</v>
       </c>
@@ -3497,7 +3636,7 @@
         <v>46545</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>24</v>
       </c>
@@ -3505,7 +3644,7 @@
         <v>46552</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>25</v>
       </c>
@@ -3513,7 +3652,7 @@
         <v>46559</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>26</v>
       </c>

</xml_diff>

<commit_message>
Mise a jour du 12-10-2026 15:42:01.56
</commit_message>
<xml_diff>
--- a/contenu/Revision Premiere.xlsx
+++ b/contenu/Revision Premiere.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maxence\Documents\Cours\Site\contenu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AF7A442-6AA2-4464-9CAE-A5342C509F80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEA1E236-2AC4-4A48-9887-FA2D343C3EA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="127">
   <si>
     <t>Préfixe</t>
   </si>
@@ -2272,9 +2272,7 @@
         <v>50</v>
       </c>
       <c r="H7" s="2"/>
-      <c r="AX7" t="s">
-        <v>107</v>
-      </c>
+      <c r="AX7"/>
     </row>
     <row r="8" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
@@ -2344,9 +2342,7 @@
       <c r="AS13" t="s">
         <v>107</v>
       </c>
-      <c r="AY13" t="s">
-        <v>107</v>
-      </c>
+      <c r="AY13"/>
     </row>
     <row r="14" spans="1:237" x14ac:dyDescent="0.3">
       <c r="A14" t="s">

</xml_diff>